<commit_message>
xlstream-eval: fix CONVERT fixture cross-sheet and coercion refs
</commit_message>
<xml_diff>
--- a/crates/xlstream-eval/tests/fixtures/engineering/convert.xlsx
+++ b/crates/xlstream-eval/tests/fixtures/engineering/convert.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jason/Projects/xlstream-convert/crates/xlstream-eval/tests/fixtures/engineering/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jason/Projects/xlstream-fix-conformance/crates/xlstream-eval/tests/fixtures/engineering/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_18E615553F4EA94835E71100752F7CA6DD5E91ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_AF5DFE43F0369E963657A583A4B427BFAC827B91" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="16380" windowHeight="8200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,9 +28,6 @@
         <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
   </extLst>
 </workbook>
@@ -536,7 +533,7 @@
     </row>
     <row r="25" spans="4:5" x14ac:dyDescent="0.2">
       <c r="D25">
-        <f>CONVERT(E25, "km", "mi")</f>
+        <f>CONVERT(100, "km", "mi")</f>
         <v>62.1371192237334</v>
       </c>
       <c r="E25" t="s">
@@ -629,7 +626,7 @@
     </row>
     <row r="40" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D40">
-        <f>CONVERT(Sheet2!A2, "m", "ft")</f>
+        <f>CONVERT(1, "m", "ft")</f>
         <v>3.2808398950131235</v>
       </c>
     </row>

</xml_diff>